<commit_message>
started loops to handle time
</commit_message>
<xml_diff>
--- a/blendmaster-backend/input/data.xlsx
+++ b/blendmaster-backend/input/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\file mappings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster-backend\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{265BB3FE-2542-45B8-9E9A-172A6CAE2B50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4395A994-2837-40BC-8F8C-FDB55E5BDE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="-3435" windowWidth="25800" windowHeight="21000" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37530" yWindow="-21780" windowWidth="51840" windowHeight="21240" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -711,6 +711,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -751,7 +752,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -783,7 +784,7 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>50000</v>
+        <v>5000</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -815,7 +816,7 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>50000</v>
+        <v>4000</v>
       </c>
       <c r="C4">
         <v>3</v>

</xml_diff>

<commit_message>
Full transactions generated for 3 periods. Inventories are still static
</commit_message>
<xml_diff>
--- a/blendmaster-backend/input/data.xlsx
+++ b/blendmaster-backend/input/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlendMaster\blendmaster-backend\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4395A994-2837-40BC-8F8C-FDB55E5BDE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD0275A-D3DA-4AA2-8260-039B8A8D6DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37530" yWindow="-21780" windowWidth="51840" windowHeight="21240" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11610" yWindow="-21660" windowWidth="25800" windowHeight="21000" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="final_input_equipment_data" sheetId="6" r:id="rId1"/>
@@ -621,19 +621,19 @@
         <v>6000</v>
       </c>
       <c r="D2">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E2">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F2">
         <v>6000</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H2">
-        <v>61.5</v>
+        <v>59</v>
       </c>
       <c r="I2">
         <v>6000</v>
@@ -710,7 +710,9 @@
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>